<commit_message>
Retorna a S/N único para taxas extras e atualiza template de parâmetros
Reverte a lógica de múltiplas colunas S/N por taxa para uma única coluna
S/N que se aplica a todas as taxas extras da unidade. Mantém taxas_extras_flag
como dict para compatibilidade interna, populando o mesmo valor S/N para
todas as taxas. Novo template Excel reflete a estrutura simplificada com
colunas A=Unidade, B=Taxa Ordinária, C=Taxa Extra S/N, D=Observações,
pré-preenchimento padrão N e instruções embutidas.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formulario_parametros.xlsx
+++ b/docs/formulario_parametros.xlsx
@@ -163,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -179,15 +179,14 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,15 +553,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -580,9 +577,7 @@
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -592,9 +587,7 @@
       </c>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -604,9 +597,7 @@
       </c>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -616,9 +607,7 @@
       </c>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -632,9 +621,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -644,9 +631,7 @@
       </c>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -747,10 +732,10 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Até 3 taxas. O nome deve ser IDÊNTICO ao nome da coluna no relatório 004A.</t>
+          <t>O nome da taxa deve ser IDÊNTICO ao nome da coluna no relatório 004A. Período: use formato mmm/aaaa (ex: jan/2026) ou selecione a data. Deixe início e fim em branco se a taxa for permanente.</t>
         </is>
       </c>
     </row>
@@ -782,34 +767,83 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
+      <c r="A21" s="2" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n"/>
+      <c r="A22" s="9" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
+      <c r="A23" s="2" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
     </row>
+    <row r="24">
+      <c r="A24" s="9" t="n"/>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n"/>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="n"/>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+    </row>
     <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>MATRIZ POR UNIDADE — Taxa Ordinária: em branco = usa padrão global. Cols C/D/E: S/N para as taxas extras declaradas nas linhas 21, 22 e 23 (respectivamente). Col F: observações livres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>MATRIZ POR UNIDADE — Taxa Ordinária: em branco = usa padrão global. Taxa Extra (col C): S = cobra todas as taxas extras declaradas acima, N = não cobra nenhuma. Col D: observações livres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Unidade</t>
@@ -820,19 +854,12 @@
           <t>Taxa Ordinária (R$)</t>
         </is>
       </c>
-      <c r="C33" s="8">
-        <f>IF(A21&lt;&gt;"",A21&amp;" (S/N)","Taxa Extra 1 (S/N)")</f>
-        <v/>
-      </c>
-      <c r="D33" s="8">
-        <f>IF(A22&lt;&gt;"",A22&amp;" (S/N)","Taxa Extra 2 (S/N)")</f>
-        <v/>
-      </c>
-      <c r="E33" s="8">
-        <f>IF(A23&lt;&gt;"",A23&amp;" (S/N)","Taxa Extra 3 (S/N)")</f>
-        <v/>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Taxa Extra? (S/N)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
@@ -841,417 +868,517 @@
     <row r="34">
       <c r="A34" s="3" t="n"/>
       <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
       <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
       <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
       <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
       <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
       <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
       <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
       <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
       <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
       <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
       <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="n"/>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
       <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="n"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
       <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="n"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
       <c r="B47" s="3" t="n"/>
-      <c r="C47" s="3" t="n"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
-      <c r="F47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
       <c r="B48" s="3" t="n"/>
-      <c r="C48" s="3" t="n"/>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="n"/>
-      <c r="F48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
       <c r="B49" s="3" t="n"/>
-      <c r="C49" s="3" t="n"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
       <c r="B50" s="3" t="n"/>
-      <c r="C50" s="3" t="n"/>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
       <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
       <c r="B52" s="3" t="n"/>
-      <c r="C52" s="3" t="n"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D52" s="3" t="n"/>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
       <c r="B53" s="3" t="n"/>
-      <c r="C53" s="3" t="n"/>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D53" s="3" t="n"/>
-      <c r="E53" s="3" t="n"/>
-      <c r="F53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
       <c r="B54" s="3" t="n"/>
-      <c r="C54" s="3" t="n"/>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
       <c r="B55" s="3" t="n"/>
-      <c r="C55" s="3" t="n"/>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
       <c r="B56" s="3" t="n"/>
-      <c r="C56" s="3" t="n"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
       <c r="B57" s="3" t="n"/>
-      <c r="C57" s="3" t="n"/>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D57" s="3" t="n"/>
-      <c r="E57" s="3" t="n"/>
-      <c r="F57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
       <c r="B58" s="3" t="n"/>
-      <c r="C58" s="3" t="n"/>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="n"/>
-      <c r="F58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
       <c r="B59" s="3" t="n"/>
-      <c r="C59" s="3" t="n"/>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D59" s="3" t="n"/>
-      <c r="E59" s="3" t="n"/>
-      <c r="F59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
       <c r="B60" s="3" t="n"/>
-      <c r="C60" s="3" t="n"/>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D60" s="3" t="n"/>
-      <c r="E60" s="3" t="n"/>
-      <c r="F60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
       <c r="B61" s="3" t="n"/>
-      <c r="C61" s="3" t="n"/>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="n"/>
-      <c r="F61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
       <c r="B62" s="3" t="n"/>
-      <c r="C62" s="3" t="n"/>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="n"/>
-      <c r="F62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
       <c r="B63" s="3" t="n"/>
-      <c r="C63" s="3" t="n"/>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D63" s="3" t="n"/>
-      <c r="E63" s="3" t="n"/>
-      <c r="F63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
       <c r="B64" s="3" t="n"/>
-      <c r="C64" s="3" t="n"/>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
-      <c r="F64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
       <c r="B65" s="3" t="n"/>
-      <c r="C65" s="3" t="n"/>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="n"/>
-      <c r="F65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
       <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
       <c r="B67" s="3" t="n"/>
-      <c r="C67" s="3" t="n"/>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
-      <c r="F67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
       <c r="B68" s="3" t="n"/>
-      <c r="C68" s="3" t="n"/>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
       <c r="B69" s="3" t="n"/>
-      <c r="C69" s="3" t="n"/>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="n"/>
-      <c r="F69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
       <c r="B70" s="3" t="n"/>
-      <c r="C70" s="3" t="n"/>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D70" s="3" t="n"/>
-      <c r="E70" s="3" t="n"/>
-      <c r="F70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
       <c r="B71" s="3" t="n"/>
-      <c r="C71" s="3" t="n"/>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D71" s="3" t="n"/>
-      <c r="E71" s="3" t="n"/>
-      <c r="F71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
       <c r="B72" s="3" t="n"/>
-      <c r="C72" s="3" t="n"/>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D72" s="3" t="n"/>
-      <c r="E72" s="3" t="n"/>
-      <c r="F72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
       <c r="B73" s="3" t="n"/>
-      <c r="C73" s="3" t="n"/>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D73" s="3" t="n"/>
-      <c r="E73" s="3" t="n"/>
-      <c r="F73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
       <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
       <c r="B75" s="3" t="n"/>
-      <c r="C75" s="3" t="n"/>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D75" s="3" t="n"/>
-      <c r="E75" s="3" t="n"/>
-      <c r="F75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
       <c r="B76" s="3" t="n"/>
-      <c r="C76" s="3" t="n"/>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D76" s="3" t="n"/>
-      <c r="E76" s="3" t="n"/>
-      <c r="F76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
       <c r="B77" s="3" t="n"/>
-      <c r="C77" s="3" t="n"/>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D77" s="3" t="n"/>
-      <c r="E77" s="3" t="n"/>
-      <c r="F77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
       <c r="B78" s="3" t="n"/>
-      <c r="C78" s="3" t="n"/>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D78" s="3" t="n"/>
-      <c r="E78" s="3" t="n"/>
-      <c r="F78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
       <c r="B79" s="3" t="n"/>
-      <c r="C79" s="3" t="n"/>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D79" s="3" t="n"/>
-      <c r="E79" s="3" t="n"/>
-      <c r="F79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
       <c r="B80" s="3" t="n"/>
-      <c r="C80" s="3" t="n"/>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D80" s="3" t="n"/>
-      <c r="E80" s="3" t="n"/>
-      <c r="F80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
       <c r="B81" s="3" t="n"/>
-      <c r="C81" s="3" t="n"/>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D81" s="3" t="n"/>
-      <c r="E81" s="3" t="n"/>
-      <c r="F81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
       <c r="B82" s="3" t="n"/>
-      <c r="C82" s="3" t="n"/>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
-      <c r="F82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
       <c r="B83" s="3" t="n"/>
-      <c r="C83" s="3" t="n"/>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D83" s="3" t="n"/>
-      <c r="E83" s="3" t="n"/>
-      <c r="F83" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>